<commit_message>
Güncel Fon ve Hisse Fiyatları
</commit_message>
<xml_diff>
--- a/piyasa_verileri.xlsx
+++ b/piyasa_verileri.xlsx
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="H2" s="1" t="n">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -554,7 +554,7 @@
       </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t>14.265,13</t>
+          <t>14.238,50</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="K4" s="1" t="inlineStr">
         <is>
-          <t>56,1744</t>
+          <t>56,1324</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="H5" s="1" t="n">
-        <v>412.5</v>
+        <v>413.75</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -683,7 +683,7 @@
       </c>
       <c r="K5" s="1" t="inlineStr">
         <is>
-          <t>77,840</t>
+          <t>77,804</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="H6" s="1" t="n">
-        <v>224.4</v>
+        <v>224.2</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="H7" s="1" t="n">
-        <v>133.8</v>
+        <v>133.6</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
       </c>
       <c r="K7" s="1" t="inlineStr">
         <is>
-          <t>107,57</t>
+          <t>108,36</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="H8" s="1" t="n">
-        <v>90.40000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
-          <t>6.743,33</t>
+          <t>6.741,29</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
         </is>
       </c>
       <c r="H9" s="1" t="n">
-        <v>429.75</v>
+        <v>429</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>0</v>
+        <v>0.203743</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="H10" s="1" t="n">
-        <v>297.75</v>
+        <v>297.25</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
         </is>
       </c>
       <c r="H11" s="1" t="n">
-        <v>72.3</v>
+        <v>72.34999999999999</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="H12" s="1" t="n">
-        <v>37.08</v>
+        <v>36.9</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="H13" s="1" t="n">
-        <v>13.84</v>
+        <v>13.83</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="K14" s="1" t="inlineStr">
         <is>
-          <t>4.313,35</t>
+          <t>4.312,80</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
         </is>
       </c>
       <c r="H15" s="1" t="n">
-        <v>47.64</v>
+        <v>47.58</v>
       </c>
     </row>
     <row r="16">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="H16" s="1" t="n">
-        <v>4612.5</v>
+        <v>4607.5</v>
       </c>
     </row>
     <row r="17">
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="H18" s="1" t="n">
-        <v>282.75</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19">
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="H19" s="1" t="n">
-        <v>82.7</v>
+        <v>82.65000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1269,7 +1269,7 @@
         </is>
       </c>
       <c r="H20" s="1" t="n">
-        <v>38.96</v>
+        <v>38.78</v>
       </c>
     </row>
     <row r="21">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="H22" s="1" t="n">
-        <v>103.1</v>
+        <v>102.8</v>
       </c>
     </row>
     <row r="23">
@@ -1368,7 +1368,7 @@
         </is>
       </c>
       <c r="H23" s="1" t="n">
-        <v>79.8</v>
+        <v>79.75</v>
       </c>
     </row>
     <row r="24">
@@ -1434,7 +1434,7 @@
         </is>
       </c>
       <c r="H25" s="1" t="n">
-        <v>59.6</v>
+        <v>58.7</v>
       </c>
     </row>
     <row r="26">
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="H26" s="1" t="n">
-        <v>94.34999999999999</v>
+        <v>94.65000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="H27" s="1" t="n">
-        <v>60.2</v>
+        <v>60.4</v>
       </c>
     </row>
     <row r="28">
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="H28" s="1" t="n">
-        <v>208.1</v>
+        <v>206.4</v>
       </c>
     </row>
     <row r="29">
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="D29" s="1" t="n">
-        <v>0</v>
+        <v>6.992015</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="H29" s="1" t="n">
-        <v>52.6</v>
+        <v>52.5</v>
       </c>
     </row>
     <row r="30">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="H30" s="1" t="n">
-        <v>494.25</v>
+        <v>489</v>
       </c>
     </row>
     <row r="31">
@@ -1632,7 +1632,7 @@
         </is>
       </c>
       <c r="H31" s="1" t="n">
-        <v>290</v>
+        <v>289.75</v>
       </c>
     </row>
     <row r="32">
@@ -1652,7 +1652,7 @@
         </is>
       </c>
       <c r="D32" s="1" t="n">
-        <v>0</v>
+        <v>16.27138</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1685,7 +1685,7 @@
         </is>
       </c>
       <c r="D33" s="1" t="n">
-        <v>0</v>
+        <v>18.650512</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
         </is>
       </c>
       <c r="H33" s="1" t="n">
-        <v>779</v>
+        <v>777.5</v>
       </c>
     </row>
     <row r="34">
@@ -1731,7 +1731,7 @@
         </is>
       </c>
       <c r="H34" s="1" t="n">
-        <v>207.4</v>
+        <v>208</v>
       </c>
     </row>
     <row r="35">
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="H35" s="1" t="n">
-        <v>115.3</v>
+        <v>115.2</v>
       </c>
     </row>
     <row r="36">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="H36" s="1" t="n">
-        <v>44.2</v>
+        <v>44.08</v>
       </c>
     </row>
     <row r="37">
@@ -1830,7 +1830,7 @@
         </is>
       </c>
       <c r="H37" s="1" t="n">
-        <v>11057.5</v>
+        <v>11035</v>
       </c>
     </row>
     <row r="38">
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="H39" s="1" t="n">
-        <v>4037.5</v>
+        <v>4032.5</v>
       </c>
     </row>
     <row r="40">
@@ -1929,7 +1929,7 @@
         </is>
       </c>
       <c r="H40" s="1" t="n">
-        <v>19.7</v>
+        <v>19.64</v>
       </c>
     </row>
     <row r="41">
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="H42" s="1" t="n">
-        <v>229.3</v>
+        <v>229</v>
       </c>
     </row>
     <row r="43">
@@ -2028,7 +2028,7 @@
         </is>
       </c>
       <c r="H43" s="1" t="n">
-        <v>22.04</v>
+        <v>22.02</v>
       </c>
     </row>
     <row r="44">
@@ -2061,7 +2061,7 @@
         </is>
       </c>
       <c r="H44" s="1" t="n">
-        <v>12.39</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="45">
@@ -2094,7 +2094,7 @@
         </is>
       </c>
       <c r="H45" s="1" t="n">
-        <v>35.1</v>
+        <v>35.24</v>
       </c>
     </row>
     <row r="46">
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="H46" s="1" t="n">
-        <v>41.04</v>
+        <v>41</v>
       </c>
     </row>
     <row r="47">
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="H50" s="1" t="n">
-        <v>270</v>
+        <v>269.75</v>
       </c>
     </row>
     <row r="51">
@@ -2325,7 +2325,7 @@
         </is>
       </c>
       <c r="H52" s="1" t="n">
-        <v>78.3</v>
+        <v>78.34999999999999</v>
       </c>
     </row>
     <row r="53">
@@ -2358,7 +2358,7 @@
         </is>
       </c>
       <c r="H53" s="1" t="n">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="54">
@@ -2391,7 +2391,7 @@
         </is>
       </c>
       <c r="H54" s="1" t="n">
-        <v>48.34</v>
+        <v>48.14</v>
       </c>
     </row>
     <row r="55">
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="H56" s="1" t="n">
-        <v>19.79</v>
+        <v>19.77</v>
       </c>
     </row>
     <row r="57">
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="H58" s="1" t="n">
-        <v>47.1</v>
+        <v>45.26</v>
       </c>
     </row>
     <row r="59">
@@ -2622,7 +2622,7 @@
         </is>
       </c>
       <c r="H61" s="1" t="n">
-        <v>439.25</v>
+        <v>438.25</v>
       </c>
     </row>
     <row r="62">
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="H62" s="1" t="n">
-        <v>34.68</v>
+        <v>34.58</v>
       </c>
     </row>
     <row r="63">
@@ -2688,7 +2688,7 @@
         </is>
       </c>
       <c r="H63" s="1" t="n">
-        <v>138.5</v>
+        <v>138.3</v>
       </c>
     </row>
     <row r="64">
@@ -2721,7 +2721,7 @@
         </is>
       </c>
       <c r="H64" s="1" t="n">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="65">
@@ -2754,7 +2754,7 @@
         </is>
       </c>
       <c r="H65" s="1" t="n">
-        <v>152.4</v>
+        <v>152</v>
       </c>
     </row>
     <row r="66">
@@ -2820,7 +2820,7 @@
         </is>
       </c>
       <c r="H67" s="1" t="n">
-        <v>20.68</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="68">
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="H68" s="1" t="n">
-        <v>328.25</v>
+        <v>329.75</v>
       </c>
     </row>
     <row r="69">
@@ -2886,7 +2886,7 @@
         </is>
       </c>
       <c r="H69" s="1" t="n">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="70">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="H70" s="1" t="n">
-        <v>200.1</v>
+        <v>199.7</v>
       </c>
     </row>
     <row r="71">
@@ -2952,7 +2952,7 @@
         </is>
       </c>
       <c r="H71" s="1" t="n">
-        <v>1387</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="72">
@@ -2985,7 +2985,7 @@
         </is>
       </c>
       <c r="H72" s="1" t="n">
-        <v>94.75</v>
+        <v>94.59999999999999</v>
       </c>
     </row>
     <row r="73">
@@ -3084,7 +3084,7 @@
         </is>
       </c>
       <c r="H75" s="1" t="n">
-        <v>24.08</v>
+        <v>24.06</v>
       </c>
     </row>
     <row r="76">
@@ -3117,7 +3117,7 @@
         </is>
       </c>
       <c r="H76" s="1" t="n">
-        <v>233.3</v>
+        <v>233.1</v>
       </c>
     </row>
     <row r="77">
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="H77" s="1" t="n">
-        <v>12.03</v>
+        <v>11.93</v>
       </c>
     </row>
     <row r="78">
@@ -3183,7 +3183,7 @@
         </is>
       </c>
       <c r="H78" s="1" t="n">
-        <v>172.8</v>
+        <v>172.6</v>
       </c>
     </row>
     <row r="79">
@@ -3216,7 +3216,7 @@
         </is>
       </c>
       <c r="H79" s="1" t="n">
-        <v>14.66</v>
+        <v>14.65</v>
       </c>
     </row>
     <row r="80">
@@ -3249,7 +3249,7 @@
         </is>
       </c>
       <c r="H80" s="1" t="n">
-        <v>94.45</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="81">
@@ -3282,7 +3282,7 @@
         </is>
       </c>
       <c r="H81" s="1" t="n">
-        <v>50.75</v>
+        <v>51.05</v>
       </c>
     </row>
     <row r="82">
@@ -3315,7 +3315,7 @@
         </is>
       </c>
       <c r="H82" s="1" t="n">
-        <v>45.22</v>
+        <v>45.24</v>
       </c>
     </row>
     <row r="83">
@@ -3381,7 +3381,7 @@
         </is>
       </c>
       <c r="H84" s="1" t="n">
-        <v>12.01</v>
+        <v>11.93</v>
       </c>
     </row>
     <row r="85">
@@ -3414,7 +3414,7 @@
         </is>
       </c>
       <c r="H85" s="1" t="n">
-        <v>504</v>
+        <v>503.5</v>
       </c>
     </row>
     <row r="86">
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="H86" s="1" t="n">
-        <v>35.22</v>
+        <v>35.2</v>
       </c>
     </row>
     <row r="87">
@@ -3480,7 +3480,7 @@
         </is>
       </c>
       <c r="H87" s="1" t="n">
-        <v>27.68</v>
+        <v>27.78</v>
       </c>
     </row>
     <row r="88">
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="H88" s="1" t="n">
-        <v>26.32</v>
+        <v>26.38</v>
       </c>
     </row>
     <row r="89">
@@ -3546,7 +3546,7 @@
         </is>
       </c>
       <c r="H89" s="1" t="n">
-        <v>223.5</v>
+        <v>223.9</v>
       </c>
     </row>
     <row r="90">
@@ -3579,7 +3579,7 @@
         </is>
       </c>
       <c r="H90" s="1" t="n">
-        <v>70.75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="91">
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="H91" s="1" t="n">
-        <v>137.5</v>
+        <v>135.8</v>
       </c>
     </row>
     <row r="92">
@@ -3645,7 +3645,7 @@
         </is>
       </c>
       <c r="H92" s="1" t="n">
-        <v>71.3</v>
+        <v>71.25</v>
       </c>
     </row>
     <row r="93">
@@ -3711,7 +3711,7 @@
         </is>
       </c>
       <c r="H94" s="1" t="n">
-        <v>1706</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="95">
@@ -3810,7 +3810,7 @@
         </is>
       </c>
       <c r="H97" s="1" t="n">
-        <v>161.5</v>
+        <v>160.4</v>
       </c>
     </row>
     <row r="98">
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="H100" s="1" t="n">
-        <v>11.28</v>
+        <v>11.27</v>
       </c>
     </row>
     <row r="101">
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="H101" s="1" t="n">
-        <v>20.88</v>
+        <v>21</v>
       </c>
     </row>
     <row r="102">
@@ -3975,7 +3975,7 @@
         </is>
       </c>
       <c r="H102" s="1" t="n">
-        <v>431.75</v>
+        <v>431.5</v>
       </c>
     </row>
     <row r="103">
@@ -4008,7 +4008,7 @@
         </is>
       </c>
       <c r="H103" s="1" t="n">
-        <v>134.1</v>
+        <v>133.6</v>
       </c>
     </row>
     <row r="104">
@@ -4041,7 +4041,7 @@
         </is>
       </c>
       <c r="H104" s="1" t="n">
-        <v>45.1</v>
+        <v>44.96</v>
       </c>
     </row>
     <row r="105">
@@ -4074,7 +4074,7 @@
         </is>
       </c>
       <c r="H105" s="1" t="n">
-        <v>221.1</v>
+        <v>219.1</v>
       </c>
     </row>
     <row r="106">
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="H106" s="1" t="n">
-        <v>537</v>
+        <v>537.5</v>
       </c>
     </row>
     <row r="107">
@@ -4140,7 +4140,7 @@
         </is>
       </c>
       <c r="H107" s="1" t="n">
-        <v>317.5</v>
+        <v>317.25</v>
       </c>
     </row>
     <row r="108">
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="H108" s="1" t="n">
-        <v>21.84</v>
+        <v>21.74</v>
       </c>
     </row>
     <row r="109">
@@ -4206,7 +4206,7 @@
         </is>
       </c>
       <c r="H109" s="1" t="n">
-        <v>61.45</v>
+        <v>61.3</v>
       </c>
     </row>
     <row r="110">
@@ -4239,7 +4239,7 @@
         </is>
       </c>
       <c r="H110" s="1" t="n">
-        <v>13.46</v>
+        <v>13.58</v>
       </c>
     </row>
     <row r="111">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="H111" s="1" t="n">
-        <v>1449</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="112">
@@ -4338,7 +4338,7 @@
         </is>
       </c>
       <c r="H113" s="1" t="n">
-        <v>76.95</v>
+        <v>76.75</v>
       </c>
     </row>
     <row r="114">
@@ -4371,7 +4371,7 @@
         </is>
       </c>
       <c r="H114" s="1" t="n">
-        <v>93.65000000000001</v>
+        <v>93.7</v>
       </c>
     </row>
     <row r="115">
@@ -4404,7 +4404,7 @@
         </is>
       </c>
       <c r="H115" s="1" t="n">
-        <v>220.9</v>
+        <v>220.1</v>
       </c>
     </row>
     <row r="116">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="H116" s="1" t="n">
-        <v>18.93</v>
+        <v>19.33</v>
       </c>
     </row>
     <row r="117">
@@ -4470,7 +4470,7 @@
         </is>
       </c>
       <c r="H117" s="1" t="n">
-        <v>60.1</v>
+        <v>60.2</v>
       </c>
     </row>
     <row r="118">
@@ -4503,7 +4503,7 @@
         </is>
       </c>
       <c r="H118" s="1" t="n">
-        <v>162.8</v>
+        <v>162.7</v>
       </c>
     </row>
     <row r="119">
@@ -4536,7 +4536,7 @@
         </is>
       </c>
       <c r="H119" s="1" t="n">
-        <v>14.35</v>
+        <v>14.42</v>
       </c>
     </row>
     <row r="120">
@@ -4569,7 +4569,7 @@
         </is>
       </c>
       <c r="H120" s="1" t="n">
-        <v>29.88</v>
+        <v>29.86</v>
       </c>
     </row>
     <row r="121">
@@ -4602,7 +4602,7 @@
         </is>
       </c>
       <c r="H121" s="1" t="n">
-        <v>16.45</v>
+        <v>16.42</v>
       </c>
     </row>
     <row r="122">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H122" s="1" t="n">
-        <v>303</v>
+        <v>303.25</v>
       </c>
     </row>
     <row r="123">
@@ -4668,7 +4668,7 @@
         </is>
       </c>
       <c r="H123" s="1" t="n">
-        <v>11.42</v>
+        <v>11.36</v>
       </c>
     </row>
     <row r="124">
@@ -4701,7 +4701,7 @@
         </is>
       </c>
       <c r="H124" s="1" t="n">
-        <v>254.25</v>
+        <v>258.5</v>
       </c>
     </row>
     <row r="125">
@@ -4734,7 +4734,7 @@
         </is>
       </c>
       <c r="H125" s="1" t="n">
-        <v>45.34</v>
+        <v>45.3</v>
       </c>
     </row>
     <row r="126">
@@ -4767,7 +4767,7 @@
         </is>
       </c>
       <c r="H126" s="1" t="n">
-        <v>183.7</v>
+        <v>182.6</v>
       </c>
     </row>
     <row r="127">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="D127" s="1" t="n">
-        <v>3.069733</v>
+        <v>3.083954</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
@@ -4800,7 +4800,7 @@
         </is>
       </c>
       <c r="H127" s="1" t="n">
-        <v>120.6</v>
+        <v>121</v>
       </c>
     </row>
     <row r="128">
@@ -4833,7 +4833,7 @@
         </is>
       </c>
       <c r="H128" s="1" t="n">
-        <v>297.5</v>
+        <v>298.25</v>
       </c>
     </row>
     <row r="129">
@@ -4866,7 +4866,7 @@
         </is>
       </c>
       <c r="H129" s="1" t="n">
-        <v>24.78</v>
+        <v>25.74</v>
       </c>
     </row>
     <row r="130">
@@ -4899,7 +4899,7 @@
         </is>
       </c>
       <c r="H130" s="1" t="n">
-        <v>36.86</v>
+        <v>36.76</v>
       </c>
     </row>
     <row r="131">
@@ -4932,7 +4932,7 @@
         </is>
       </c>
       <c r="H131" s="1" t="n">
-        <v>226.5</v>
+        <v>234.4</v>
       </c>
     </row>
     <row r="132">
@@ -4965,7 +4965,7 @@
         </is>
       </c>
       <c r="H132" s="1" t="n">
-        <v>36.16</v>
+        <v>35.88</v>
       </c>
     </row>
     <row r="133">
@@ -4985,7 +4985,7 @@
         </is>
       </c>
       <c r="D133" s="1" t="n">
-        <v>2.675759</v>
+        <v>2.675763</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
         </is>
       </c>
       <c r="H133" s="1" t="n">
-        <v>60.8</v>
+        <v>60.85</v>
       </c>
     </row>
     <row r="134">
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="H134" s="1" t="n">
-        <v>106.6</v>
+        <v>107</v>
       </c>
     </row>
     <row r="135">
@@ -5064,7 +5064,7 @@
         </is>
       </c>
       <c r="H135" s="1" t="n">
-        <v>71.59999999999999</v>
+        <v>71.5</v>
       </c>
     </row>
     <row r="136">
@@ -5097,7 +5097,7 @@
         </is>
       </c>
       <c r="H136" s="1" t="n">
-        <v>1.33</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="137">
@@ -5130,7 +5130,7 @@
         </is>
       </c>
       <c r="H137" s="1" t="n">
-        <v>94.2</v>
+        <v>95.7</v>
       </c>
     </row>
     <row r="138">
@@ -5163,7 +5163,7 @@
         </is>
       </c>
       <c r="H138" s="1" t="n">
-        <v>13.7</v>
+        <v>13.72</v>
       </c>
     </row>
     <row r="139">
@@ -5196,7 +5196,7 @@
         </is>
       </c>
       <c r="H139" s="1" t="n">
-        <v>78.95</v>
+        <v>78.90000000000001</v>
       </c>
     </row>
     <row r="140">
@@ -5229,7 +5229,7 @@
         </is>
       </c>
       <c r="H140" s="1" t="n">
-        <v>62</v>
+        <v>61.25</v>
       </c>
     </row>
     <row r="141">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="H141" s="1" t="n">
-        <v>150.9</v>
+        <v>151.1</v>
       </c>
     </row>
     <row r="142">
@@ -5295,7 +5295,7 @@
         </is>
       </c>
       <c r="H142" s="1" t="n">
-        <v>10.07</v>
+        <v>10.04</v>
       </c>
     </row>
     <row r="143">
@@ -5394,7 +5394,7 @@
         </is>
       </c>
       <c r="H145" s="1" t="n">
-        <v>78.3</v>
+        <v>78.05</v>
       </c>
     </row>
     <row r="146">
@@ -5427,7 +5427,7 @@
         </is>
       </c>
       <c r="H146" s="1" t="n">
-        <v>140.1</v>
+        <v>139.6</v>
       </c>
     </row>
     <row r="147">
@@ -5460,7 +5460,7 @@
         </is>
       </c>
       <c r="H147" s="1" t="n">
-        <v>8.93</v>
+        <v>8.869999999999999</v>
       </c>
     </row>
     <row r="148">
@@ -5493,7 +5493,7 @@
         </is>
       </c>
       <c r="H148" s="1" t="n">
-        <v>11930</v>
+        <v>11947.5</v>
       </c>
     </row>
     <row r="149">
@@ -5526,7 +5526,7 @@
         </is>
       </c>
       <c r="H149" s="1" t="n">
-        <v>23.24</v>
+        <v>23.18</v>
       </c>
     </row>
     <row r="150">
@@ -5559,7 +5559,7 @@
         </is>
       </c>
       <c r="H150" s="1" t="n">
-        <v>54.95</v>
+        <v>55.2</v>
       </c>
     </row>
     <row r="151">
@@ -5592,7 +5592,7 @@
         </is>
       </c>
       <c r="H151" s="1" t="n">
-        <v>3.79</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="152">
@@ -5625,7 +5625,7 @@
         </is>
       </c>
       <c r="H152" s="1" t="n">
-        <v>43.06</v>
+        <v>43.24</v>
       </c>
     </row>
     <row r="153">
@@ -5658,7 +5658,7 @@
         </is>
       </c>
       <c r="H153" s="1" t="n">
-        <v>8.19</v>
+        <v>8.119999999999999</v>
       </c>
     </row>
     <row r="154">
@@ -5724,7 +5724,7 @@
         </is>
       </c>
       <c r="H155" s="1" t="n">
-        <v>177.2</v>
+        <v>178.9</v>
       </c>
     </row>
     <row r="156">
@@ -5757,7 +5757,7 @@
         </is>
       </c>
       <c r="H156" s="1" t="n">
-        <v>3.15</v>
+        <v>3.16</v>
       </c>
     </row>
     <row r="157">
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="H157" s="1" t="n">
-        <v>31.76</v>
+        <v>31.82</v>
       </c>
     </row>
     <row r="158">
@@ -5823,7 +5823,7 @@
         </is>
       </c>
       <c r="H158" s="1" t="n">
-        <v>38.12</v>
+        <v>38.3</v>
       </c>
     </row>
     <row r="159">
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="H159" s="1" t="n">
-        <v>37.22</v>
+        <v>37.1</v>
       </c>
     </row>
     <row r="160">
@@ -5889,7 +5889,7 @@
         </is>
       </c>
       <c r="H160" s="1" t="n">
-        <v>4350</v>
+        <v>4300</v>
       </c>
     </row>
     <row r="161">
@@ -5922,7 +5922,7 @@
         </is>
       </c>
       <c r="H161" s="1" t="n">
-        <v>105.5</v>
+        <v>107</v>
       </c>
     </row>
     <row r="162">
@@ -5955,7 +5955,7 @@
         </is>
       </c>
       <c r="H162" s="1" t="n">
-        <v>41.24</v>
+        <v>41.12</v>
       </c>
     </row>
     <row r="163">
@@ -5988,7 +5988,7 @@
         </is>
       </c>
       <c r="H163" s="1" t="n">
-        <v>37.5</v>
+        <v>37.4</v>
       </c>
     </row>
     <row r="164">
@@ -6054,7 +6054,7 @@
         </is>
       </c>
       <c r="H165" s="1" t="n">
-        <v>1705</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="166">
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="H166" s="1" t="n">
-        <v>13.02</v>
+        <v>13.03</v>
       </c>
     </row>
     <row r="167">
@@ -6120,7 +6120,7 @@
         </is>
       </c>
       <c r="H167" s="1" t="n">
-        <v>6442.5</v>
+        <v>6315</v>
       </c>
     </row>
     <row r="168">
@@ -6153,7 +6153,7 @@
         </is>
       </c>
       <c r="H168" s="1" t="n">
-        <v>26.52</v>
+        <v>26.44</v>
       </c>
     </row>
     <row r="169">
@@ -6186,7 +6186,7 @@
         </is>
       </c>
       <c r="H169" s="1" t="n">
-        <v>234.4</v>
+        <v>235.8</v>
       </c>
     </row>
     <row r="170">
@@ -6219,7 +6219,7 @@
         </is>
       </c>
       <c r="H170" s="1" t="n">
-        <v>37.88</v>
+        <v>38.08</v>
       </c>
     </row>
     <row r="171">
@@ -6252,7 +6252,7 @@
         </is>
       </c>
       <c r="H171" s="1" t="n">
-        <v>2.9</v>
+        <v>2.91</v>
       </c>
     </row>
     <row r="172">
@@ -6285,7 +6285,7 @@
         </is>
       </c>
       <c r="H172" s="1" t="n">
-        <v>21.64</v>
+        <v>21.44</v>
       </c>
     </row>
     <row r="173">
@@ -6318,7 +6318,7 @@
         </is>
       </c>
       <c r="H173" s="1" t="n">
-        <v>17.13</v>
+        <v>17.14</v>
       </c>
     </row>
     <row r="174">
@@ -6338,7 +6338,7 @@
         </is>
       </c>
       <c r="D174" s="1" t="n">
-        <v>4.405776</v>
+        <v>4.408489</v>
       </c>
       <c r="F174" t="inlineStr">
         <is>
@@ -6351,7 +6351,7 @@
         </is>
       </c>
       <c r="H174" s="1" t="n">
-        <v>106.6</v>
+        <v>107.3</v>
       </c>
     </row>
     <row r="175">
@@ -6384,7 +6384,7 @@
         </is>
       </c>
       <c r="H175" s="1" t="n">
-        <v>4.26</v>
+        <v>4.28</v>
       </c>
     </row>
     <row r="176">
@@ -6417,7 +6417,7 @@
         </is>
       </c>
       <c r="H176" s="1" t="n">
-        <v>6.91</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="177">
@@ -6450,7 +6450,7 @@
         </is>
       </c>
       <c r="H177" s="1" t="n">
-        <v>25.06</v>
+        <v>25.08</v>
       </c>
     </row>
     <row r="178">
@@ -6483,7 +6483,7 @@
         </is>
       </c>
       <c r="H178" s="1" t="n">
-        <v>15.59</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="179">
@@ -6516,7 +6516,7 @@
         </is>
       </c>
       <c r="H179" s="1" t="n">
-        <v>28.46</v>
+        <v>28.44</v>
       </c>
     </row>
     <row r="180">
@@ -6549,7 +6549,7 @@
         </is>
       </c>
       <c r="H180" s="1" t="n">
-        <v>4.4</v>
+        <v>4.39</v>
       </c>
     </row>
     <row r="181">
@@ -6582,7 +6582,7 @@
         </is>
       </c>
       <c r="H181" s="1" t="n">
-        <v>22.2</v>
+        <v>22.08</v>
       </c>
     </row>
     <row r="182">
@@ -6615,7 +6615,7 @@
         </is>
       </c>
       <c r="H182" s="1" t="n">
-        <v>18.73</v>
+        <v>18.82</v>
       </c>
     </row>
     <row r="183">
@@ -6648,7 +6648,7 @@
         </is>
       </c>
       <c r="H183" s="1" t="n">
-        <v>176.2</v>
+        <v>175.4</v>
       </c>
     </row>
     <row r="184">
@@ -6681,7 +6681,7 @@
         </is>
       </c>
       <c r="H184" s="1" t="n">
-        <v>10.25</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="185">
@@ -6747,7 +6747,7 @@
         </is>
       </c>
       <c r="H186" s="1" t="n">
-        <v>114.9</v>
+        <v>114.8</v>
       </c>
     </row>
     <row r="187">
@@ -6780,7 +6780,7 @@
         </is>
       </c>
       <c r="H187" s="1" t="n">
-        <v>128</v>
+        <v>127.8</v>
       </c>
     </row>
     <row r="188">
@@ -6813,7 +6813,7 @@
         </is>
       </c>
       <c r="H188" s="1" t="n">
-        <v>5.36</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="189">
@@ -6846,7 +6846,7 @@
         </is>
       </c>
       <c r="H189" s="1" t="n">
-        <v>4120</v>
+        <v>4097.5</v>
       </c>
     </row>
     <row r="190">
@@ -6879,7 +6879,7 @@
         </is>
       </c>
       <c r="H190" s="1" t="n">
-        <v>10.72</v>
+        <v>10.75</v>
       </c>
     </row>
     <row r="191">
@@ -6912,7 +6912,7 @@
         </is>
       </c>
       <c r="H191" s="1" t="n">
-        <v>152.9</v>
+        <v>152.5</v>
       </c>
     </row>
     <row r="192">
@@ -6945,7 +6945,7 @@
         </is>
       </c>
       <c r="H192" s="1" t="n">
-        <v>33.04</v>
+        <v>32.84</v>
       </c>
     </row>
     <row r="193">
@@ -6978,7 +6978,7 @@
         </is>
       </c>
       <c r="H193" s="1" t="n">
-        <v>8.369999999999999</v>
+        <v>8.32</v>
       </c>
     </row>
     <row r="194">
@@ -7011,7 +7011,7 @@
         </is>
       </c>
       <c r="H194" s="1" t="n">
-        <v>3.96</v>
+        <v>3.94</v>
       </c>
     </row>
     <row r="195">
@@ -7044,7 +7044,7 @@
         </is>
       </c>
       <c r="H195" s="1" t="n">
-        <v>52.1</v>
+        <v>52.4</v>
       </c>
     </row>
     <row r="196">
@@ -7077,7 +7077,7 @@
         </is>
       </c>
       <c r="H196" s="1" t="n">
-        <v>44.96</v>
+        <v>45.1</v>
       </c>
     </row>
     <row r="197">
@@ -7110,7 +7110,7 @@
         </is>
       </c>
       <c r="H197" s="1" t="n">
-        <v>38.34</v>
+        <v>38.32</v>
       </c>
     </row>
     <row r="198">
@@ -7143,7 +7143,7 @@
         </is>
       </c>
       <c r="H198" s="1" t="n">
-        <v>64.05</v>
+        <v>63.55</v>
       </c>
     </row>
     <row r="199">
@@ -7176,7 +7176,7 @@
         </is>
       </c>
       <c r="H199" s="1" t="n">
-        <v>1.03</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="200">
@@ -7209,7 +7209,7 @@
         </is>
       </c>
       <c r="H200" s="1" t="n">
-        <v>84.95</v>
+        <v>84.34999999999999</v>
       </c>
     </row>
     <row r="201">
@@ -7242,7 +7242,7 @@
         </is>
       </c>
       <c r="H201" s="1" t="n">
-        <v>36.92</v>
+        <v>36.98</v>
       </c>
     </row>
     <row r="202">
@@ -7308,7 +7308,7 @@
         </is>
       </c>
       <c r="H203" s="1" t="n">
-        <v>14.48</v>
+        <v>14.17</v>
       </c>
     </row>
     <row r="204">
@@ -7341,7 +7341,7 @@
         </is>
       </c>
       <c r="H204" s="1" t="n">
-        <v>19.11</v>
+        <v>19.12</v>
       </c>
     </row>
     <row r="205">
@@ -7374,7 +7374,7 @@
         </is>
       </c>
       <c r="H205" s="1" t="n">
-        <v>139</v>
+        <v>139.1</v>
       </c>
     </row>
     <row r="206">
@@ -7407,7 +7407,7 @@
         </is>
       </c>
       <c r="H206" s="1" t="n">
-        <v>20.24</v>
+        <v>20.28</v>
       </c>
     </row>
     <row r="207">
@@ -7473,7 +7473,7 @@
         </is>
       </c>
       <c r="H208" s="1" t="n">
-        <v>45.4</v>
+        <v>47.08</v>
       </c>
     </row>
     <row r="209">
@@ -7506,7 +7506,7 @@
         </is>
       </c>
       <c r="H209" s="1" t="n">
-        <v>9.92</v>
+        <v>9.91</v>
       </c>
     </row>
     <row r="210">
@@ -7539,7 +7539,7 @@
         </is>
       </c>
       <c r="H210" s="1" t="n">
-        <v>49.08</v>
+        <v>48.84</v>
       </c>
     </row>
     <row r="211">
@@ -7559,7 +7559,7 @@
         </is>
       </c>
       <c r="D211" s="1" t="n">
-        <v>0</v>
+        <v>12.595743</v>
       </c>
       <c r="F211" t="inlineStr">
         <is>
@@ -7572,7 +7572,7 @@
         </is>
       </c>
       <c r="H211" s="1" t="n">
-        <v>3.18</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="212">
@@ -7605,7 +7605,7 @@
         </is>
       </c>
       <c r="H212" s="1" t="n">
-        <v>31.28</v>
+        <v>31.32</v>
       </c>
     </row>
     <row r="213">
@@ -7638,7 +7638,7 @@
         </is>
       </c>
       <c r="H213" s="1" t="n">
-        <v>45.64</v>
+        <v>45.54</v>
       </c>
     </row>
     <row r="214">
@@ -7671,7 +7671,7 @@
         </is>
       </c>
       <c r="H214" s="1" t="n">
-        <v>22.74</v>
+        <v>22.72</v>
       </c>
     </row>
     <row r="215">
@@ -7704,7 +7704,7 @@
         </is>
       </c>
       <c r="H215" s="1" t="n">
-        <v>2.86</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="216">
@@ -7737,7 +7737,7 @@
         </is>
       </c>
       <c r="H216" s="1" t="n">
-        <v>2.44</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="217">
@@ -7803,7 +7803,7 @@
         </is>
       </c>
       <c r="H218" s="1" t="n">
-        <v>26.38</v>
+        <v>26.34</v>
       </c>
     </row>
     <row r="219">
@@ -7902,7 +7902,7 @@
         </is>
       </c>
       <c r="H221" s="1" t="n">
-        <v>160.6</v>
+        <v>160</v>
       </c>
     </row>
     <row r="222">
@@ -7935,7 +7935,7 @@
         </is>
       </c>
       <c r="H222" s="1" t="n">
-        <v>4.04</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="223">
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="H223" s="1" t="n">
-        <v>23.02</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="224">
@@ -8001,7 +8001,7 @@
         </is>
       </c>
       <c r="H224" s="1" t="n">
-        <v>137.2</v>
+        <v>135.7</v>
       </c>
     </row>
     <row r="225">
@@ -8034,7 +8034,7 @@
         </is>
       </c>
       <c r="H225" s="1" t="n">
-        <v>96.7</v>
+        <v>97.45</v>
       </c>
     </row>
     <row r="226">
@@ -8067,7 +8067,7 @@
         </is>
       </c>
       <c r="H226" s="1" t="n">
-        <v>16.54</v>
+        <v>16.51</v>
       </c>
     </row>
     <row r="227">
@@ -8100,7 +8100,7 @@
         </is>
       </c>
       <c r="H227" s="1" t="n">
-        <v>22.28</v>
+        <v>22.32</v>
       </c>
     </row>
     <row r="228">
@@ -8133,7 +8133,7 @@
         </is>
       </c>
       <c r="H228" s="1" t="n">
-        <v>11.44</v>
+        <v>11.55</v>
       </c>
     </row>
     <row r="229">
@@ -8166,7 +8166,7 @@
         </is>
       </c>
       <c r="H229" s="1" t="n">
-        <v>9.539999999999999</v>
+        <v>9.380000000000001</v>
       </c>
     </row>
     <row r="230">
@@ -8199,7 +8199,7 @@
         </is>
       </c>
       <c r="H230" s="1" t="n">
-        <v>34.28</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="231">
@@ -8232,7 +8232,7 @@
         </is>
       </c>
       <c r="H231" s="1" t="n">
-        <v>14.11</v>
+        <v>14.16</v>
       </c>
     </row>
     <row r="232">
@@ -8265,7 +8265,7 @@
         </is>
       </c>
       <c r="H232" s="1" t="n">
-        <v>110.6</v>
+        <v>110.8</v>
       </c>
     </row>
     <row r="233">
@@ -8298,7 +8298,7 @@
         </is>
       </c>
       <c r="H233" s="1" t="n">
-        <v>2.82</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="234">
@@ -8331,7 +8331,7 @@
         </is>
       </c>
       <c r="H234" s="1" t="n">
-        <v>33.06</v>
+        <v>33.42</v>
       </c>
     </row>
     <row r="235">
@@ -8364,7 +8364,7 @@
         </is>
       </c>
       <c r="H235" s="1" t="n">
-        <v>65.95</v>
+        <v>65.55</v>
       </c>
     </row>
     <row r="236">
@@ -8397,7 +8397,7 @@
         </is>
       </c>
       <c r="H236" s="1" t="n">
-        <v>525</v>
+        <v>530.5</v>
       </c>
     </row>
     <row r="237">
@@ -8430,7 +8430,7 @@
         </is>
       </c>
       <c r="H237" s="1" t="n">
-        <v>10.02</v>
+        <v>10.04</v>
       </c>
     </row>
     <row r="238">
@@ -8463,7 +8463,7 @@
         </is>
       </c>
       <c r="H238" s="1" t="n">
-        <v>27.12</v>
+        <v>26.98</v>
       </c>
     </row>
     <row r="239">
@@ -8496,7 +8496,7 @@
         </is>
       </c>
       <c r="H239" s="1" t="n">
-        <v>17.84</v>
+        <v>17.83</v>
       </c>
     </row>
     <row r="240">
@@ -8529,7 +8529,7 @@
         </is>
       </c>
       <c r="H240" s="1" t="n">
-        <v>424.25</v>
+        <v>424.5</v>
       </c>
     </row>
     <row r="241">
@@ -8562,7 +8562,7 @@
         </is>
       </c>
       <c r="H241" s="1" t="n">
-        <v>66.55</v>
+        <v>66.8</v>
       </c>
     </row>
     <row r="242">
@@ -8595,7 +8595,7 @@
         </is>
       </c>
       <c r="H242" s="1" t="n">
-        <v>28.12</v>
+        <v>27.84</v>
       </c>
     </row>
     <row r="243">
@@ -8628,7 +8628,7 @@
         </is>
       </c>
       <c r="H243" s="1" t="n">
-        <v>34.76</v>
+        <v>34.74</v>
       </c>
     </row>
     <row r="244">
@@ -8661,7 +8661,7 @@
         </is>
       </c>
       <c r="H244" s="1" t="n">
-        <v>60.2</v>
+        <v>59.85</v>
       </c>
     </row>
     <row r="245">
@@ -8694,7 +8694,7 @@
         </is>
       </c>
       <c r="H245" s="1" t="n">
-        <v>6.97</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="246">
@@ -8760,7 +8760,7 @@
         </is>
       </c>
       <c r="H247" s="1" t="n">
-        <v>136.7</v>
+        <v>136.5</v>
       </c>
     </row>
     <row r="248">
@@ -8793,7 +8793,7 @@
         </is>
       </c>
       <c r="H248" s="1" t="n">
-        <v>11.3</v>
+        <v>11.25</v>
       </c>
     </row>
     <row r="249">
@@ -8826,7 +8826,7 @@
         </is>
       </c>
       <c r="H249" s="1" t="n">
-        <v>62.95</v>
+        <v>63</v>
       </c>
     </row>
     <row r="250">
@@ -8859,7 +8859,7 @@
         </is>
       </c>
       <c r="H250" s="1" t="n">
-        <v>12.18</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="251">
@@ -8892,7 +8892,7 @@
         </is>
       </c>
       <c r="H251" s="1" t="n">
-        <v>192.3</v>
+        <v>196.1</v>
       </c>
     </row>
     <row r="252">
@@ -8925,7 +8925,7 @@
         </is>
       </c>
       <c r="H252" s="1" t="n">
-        <v>33.1</v>
+        <v>32.98</v>
       </c>
     </row>
     <row r="253">
@@ -8958,7 +8958,7 @@
         </is>
       </c>
       <c r="H253" s="1" t="n">
-        <v>35.24</v>
+        <v>35.12</v>
       </c>
     </row>
     <row r="254">
@@ -8991,7 +8991,7 @@
         </is>
       </c>
       <c r="H254" s="1" t="n">
-        <v>286.25</v>
+        <v>286.5</v>
       </c>
     </row>
     <row r="255">
@@ -9057,7 +9057,7 @@
         </is>
       </c>
       <c r="H256" s="1" t="n">
-        <v>8.48</v>
+        <v>8.449999999999999</v>
       </c>
     </row>
     <row r="257">
@@ -9090,7 +9090,7 @@
         </is>
       </c>
       <c r="H257" s="1" t="n">
-        <v>11.02</v>
+        <v>11</v>
       </c>
     </row>
     <row r="258">
@@ -9123,7 +9123,7 @@
         </is>
       </c>
       <c r="H258" s="1" t="n">
-        <v>67.09999999999999</v>
+        <v>66.8</v>
       </c>
     </row>
     <row r="259">
@@ -9156,7 +9156,7 @@
         </is>
       </c>
       <c r="H259" s="1" t="n">
-        <v>19.03</v>
+        <v>19</v>
       </c>
     </row>
     <row r="260">
@@ -9222,7 +9222,7 @@
         </is>
       </c>
       <c r="H261" s="1" t="n">
-        <v>70.3</v>
+        <v>70.2</v>
       </c>
     </row>
     <row r="262">
@@ -9255,7 +9255,7 @@
         </is>
       </c>
       <c r="H262" s="1" t="n">
-        <v>24.46</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="263">
@@ -9288,7 +9288,7 @@
         </is>
       </c>
       <c r="H263" s="1" t="n">
-        <v>24.44</v>
+        <v>24.64</v>
       </c>
     </row>
     <row r="264">
@@ -9321,7 +9321,7 @@
         </is>
       </c>
       <c r="H264" s="1" t="n">
-        <v>82.05</v>
+        <v>83</v>
       </c>
     </row>
     <row r="265">
@@ -9354,7 +9354,7 @@
         </is>
       </c>
       <c r="H265" s="1" t="n">
-        <v>5.68</v>
+        <v>5.67</v>
       </c>
     </row>
     <row r="266">
@@ -9420,7 +9420,7 @@
         </is>
       </c>
       <c r="H267" s="1" t="n">
-        <v>22.86</v>
+        <v>22.98</v>
       </c>
     </row>
     <row r="268">
@@ -9486,7 +9486,7 @@
         </is>
       </c>
       <c r="H269" s="1" t="n">
-        <v>18.99</v>
+        <v>18.85</v>
       </c>
     </row>
     <row r="270">
@@ -9519,7 +9519,7 @@
         </is>
       </c>
       <c r="H270" s="1" t="n">
-        <v>245.2</v>
+        <v>244.9</v>
       </c>
     </row>
     <row r="271">
@@ -9552,7 +9552,7 @@
         </is>
       </c>
       <c r="H271" s="1" t="n">
-        <v>13.72</v>
+        <v>13.74</v>
       </c>
     </row>
     <row r="272">
@@ -9585,7 +9585,7 @@
         </is>
       </c>
       <c r="H272" s="1" t="n">
-        <v>5.6</v>
+        <v>5.61</v>
       </c>
     </row>
     <row r="273">
@@ -9651,7 +9651,7 @@
         </is>
       </c>
       <c r="H274" s="1" t="n">
-        <v>11.72</v>
+        <v>11.71</v>
       </c>
     </row>
     <row r="275">
@@ -9750,7 +9750,7 @@
         </is>
       </c>
       <c r="H277" s="1" t="n">
-        <v>25.06</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="278">
@@ -9783,7 +9783,7 @@
         </is>
       </c>
       <c r="H278" s="1" t="n">
-        <v>31</v>
+        <v>30.96</v>
       </c>
     </row>
     <row r="279">
@@ -9816,7 +9816,7 @@
         </is>
       </c>
       <c r="H279" s="1" t="n">
-        <v>7.63</v>
+        <v>7.61</v>
       </c>
     </row>
     <row r="280">
@@ -9849,7 +9849,7 @@
         </is>
       </c>
       <c r="H280" s="1" t="n">
-        <v>12.94</v>
+        <v>12.95</v>
       </c>
     </row>
     <row r="281">
@@ -9948,7 +9948,7 @@
         </is>
       </c>
       <c r="H283" s="1" t="n">
-        <v>31.24</v>
+        <v>31.46</v>
       </c>
     </row>
     <row r="284">
@@ -9981,7 +9981,7 @@
         </is>
       </c>
       <c r="H284" s="1" t="n">
-        <v>6.46</v>
+        <v>6.45</v>
       </c>
     </row>
     <row r="285">
@@ -10014,7 +10014,7 @@
         </is>
       </c>
       <c r="H285" s="1" t="n">
-        <v>1012</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="286">
@@ -10047,7 +10047,7 @@
         </is>
       </c>
       <c r="H286" s="1" t="n">
-        <v>72</v>
+        <v>72.05</v>
       </c>
     </row>
     <row r="287">
@@ -10080,7 +10080,7 @@
         </is>
       </c>
       <c r="H287" s="1" t="n">
-        <v>32.18</v>
+        <v>32.44</v>
       </c>
     </row>
     <row r="288">
@@ -10146,7 +10146,7 @@
         </is>
       </c>
       <c r="H289" s="1" t="n">
-        <v>50.4</v>
+        <v>50.1</v>
       </c>
     </row>
     <row r="290">
@@ -10179,7 +10179,7 @@
         </is>
       </c>
       <c r="H290" s="1" t="n">
-        <v>44.9</v>
+        <v>45.34</v>
       </c>
     </row>
     <row r="291">
@@ -10212,7 +10212,7 @@
         </is>
       </c>
       <c r="H291" s="1" t="n">
-        <v>2.45</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="292">
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="H293" s="1" t="n">
-        <v>15.59</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="294">
@@ -10311,7 +10311,7 @@
         </is>
       </c>
       <c r="H294" s="1" t="n">
-        <v>764.5</v>
+        <v>763</v>
       </c>
     </row>
     <row r="295">
@@ -10344,7 +10344,7 @@
         </is>
       </c>
       <c r="H295" s="1" t="n">
-        <v>11.38</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="296">
@@ -10410,7 +10410,7 @@
         </is>
       </c>
       <c r="H297" s="1" t="n">
-        <v>30.24</v>
+        <v>30.2</v>
       </c>
     </row>
     <row r="298">
@@ -10443,7 +10443,7 @@
         </is>
       </c>
       <c r="H298" s="1" t="n">
-        <v>118.4</v>
+        <v>118.2</v>
       </c>
     </row>
     <row r="299">
@@ -10476,7 +10476,7 @@
         </is>
       </c>
       <c r="H299" s="1" t="n">
-        <v>3.74</v>
+        <v>3.73</v>
       </c>
     </row>
     <row r="300">
@@ -10509,7 +10509,7 @@
         </is>
       </c>
       <c r="H300" s="1" t="n">
-        <v>10.3</v>
+        <v>10.32</v>
       </c>
     </row>
     <row r="301">
@@ -10575,7 +10575,7 @@
         </is>
       </c>
       <c r="H302" s="1" t="n">
-        <v>23.22</v>
+        <v>23.3</v>
       </c>
     </row>
     <row r="303">
@@ -10608,7 +10608,7 @@
         </is>
       </c>
       <c r="H303" s="1" t="n">
-        <v>52.8</v>
+        <v>52.85</v>
       </c>
     </row>
     <row r="304">
@@ -10641,7 +10641,7 @@
         </is>
       </c>
       <c r="H304" s="1" t="n">
-        <v>40.38</v>
+        <v>40.4</v>
       </c>
     </row>
     <row r="305">
@@ -10674,7 +10674,7 @@
         </is>
       </c>
       <c r="H305" s="1" t="n">
-        <v>11.17</v>
+        <v>11.19</v>
       </c>
     </row>
     <row r="306">
@@ -10707,7 +10707,7 @@
         </is>
       </c>
       <c r="H306" s="1" t="n">
-        <v>367.75</v>
+        <v>363</v>
       </c>
     </row>
     <row r="307">
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="H307" s="1" t="n">
-        <v>1.82</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="308">
@@ -10773,7 +10773,7 @@
         </is>
       </c>
       <c r="H308" s="1" t="n">
-        <v>16.73</v>
+        <v>16.81</v>
       </c>
     </row>
     <row r="309">
@@ -10806,7 +10806,7 @@
         </is>
       </c>
       <c r="H309" s="1" t="n">
-        <v>20.2</v>
+        <v>20.28</v>
       </c>
     </row>
     <row r="310">
@@ -10872,7 +10872,7 @@
         </is>
       </c>
       <c r="H311" s="1" t="n">
-        <v>23.26</v>
+        <v>23.3</v>
       </c>
     </row>
     <row r="312">
@@ -10905,7 +10905,7 @@
         </is>
       </c>
       <c r="H312" s="1" t="n">
-        <v>4.14</v>
+        <v>4.13</v>
       </c>
     </row>
     <row r="313">
@@ -10938,7 +10938,7 @@
         </is>
       </c>
       <c r="H313" s="1" t="n">
-        <v>280.25</v>
+        <v>279.75</v>
       </c>
     </row>
     <row r="314">
@@ -10971,7 +10971,7 @@
         </is>
       </c>
       <c r="H314" s="1" t="n">
-        <v>25.22</v>
+        <v>25.24</v>
       </c>
     </row>
     <row r="315">
@@ -11037,7 +11037,7 @@
         </is>
       </c>
       <c r="H316" s="1" t="n">
-        <v>31.42</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="317">
@@ -11070,7 +11070,7 @@
         </is>
       </c>
       <c r="H317" s="1" t="n">
-        <v>10.63</v>
+        <v>10.73</v>
       </c>
     </row>
     <row r="318">
@@ -11103,7 +11103,7 @@
         </is>
       </c>
       <c r="H318" s="1" t="n">
-        <v>6.67</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="319">
@@ -11136,7 +11136,7 @@
         </is>
       </c>
       <c r="H319" s="1" t="n">
-        <v>4.69</v>
+        <v>4.64</v>
       </c>
     </row>
     <row r="320">
@@ -11235,7 +11235,7 @@
         </is>
       </c>
       <c r="H322" s="1" t="n">
-        <v>15.91</v>
+        <v>15.86</v>
       </c>
     </row>
     <row r="323">
@@ -11268,7 +11268,7 @@
         </is>
       </c>
       <c r="H323" s="1" t="n">
-        <v>8.039999999999999</v>
+        <v>8.029999999999999</v>
       </c>
     </row>
     <row r="324">
@@ -11367,7 +11367,7 @@
         </is>
       </c>
       <c r="H326" s="1" t="n">
-        <v>37.12</v>
+        <v>37.04</v>
       </c>
     </row>
     <row r="327">
@@ -11400,7 +11400,7 @@
         </is>
       </c>
       <c r="H327" s="1" t="n">
-        <v>3.43</v>
+        <v>3.44</v>
       </c>
     </row>
     <row r="328">
@@ -11433,7 +11433,7 @@
         </is>
       </c>
       <c r="H328" s="1" t="n">
-        <v>9.789999999999999</v>
+        <v>9.779999999999999</v>
       </c>
     </row>
     <row r="329">
@@ -11466,7 +11466,7 @@
         </is>
       </c>
       <c r="H329" s="1" t="n">
-        <v>18.12</v>
+        <v>18.21</v>
       </c>
     </row>
     <row r="330">
@@ -11499,7 +11499,7 @@
         </is>
       </c>
       <c r="H330" s="1" t="n">
-        <v>72.40000000000001</v>
+        <v>72.59999999999999</v>
       </c>
     </row>
     <row r="331">
@@ -11532,7 +11532,7 @@
         </is>
       </c>
       <c r="H331" s="1" t="n">
-        <v>10.3</v>
+        <v>10.31</v>
       </c>
     </row>
     <row r="332">
@@ -11565,7 +11565,7 @@
         </is>
       </c>
       <c r="H332" s="1" t="n">
-        <v>6.49</v>
+        <v>6.46</v>
       </c>
     </row>
     <row r="333">
@@ -11598,7 +11598,7 @@
         </is>
       </c>
       <c r="H333" s="1" t="n">
-        <v>96.09999999999999</v>
+        <v>97.3</v>
       </c>
     </row>
     <row r="334">
@@ -11631,7 +11631,7 @@
         </is>
       </c>
       <c r="H334" s="1" t="n">
-        <v>8.16</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="335">
@@ -11664,7 +11664,7 @@
         </is>
       </c>
       <c r="H335" s="1" t="n">
-        <v>7.95</v>
+        <v>7.92</v>
       </c>
     </row>
     <row r="336">
@@ -11697,7 +11697,7 @@
         </is>
       </c>
       <c r="H336" s="1" t="n">
-        <v>29.9</v>
+        <v>30.34</v>
       </c>
     </row>
     <row r="337">
@@ -11730,7 +11730,7 @@
         </is>
       </c>
       <c r="H337" s="1" t="n">
-        <v>74.5</v>
+        <v>76.34999999999999</v>
       </c>
     </row>
     <row r="338">
@@ -11796,7 +11796,7 @@
         </is>
       </c>
       <c r="H339" s="1" t="n">
-        <v>30.4</v>
+        <v>30.62</v>
       </c>
     </row>
     <row r="340">
@@ -11829,7 +11829,7 @@
         </is>
       </c>
       <c r="H340" s="1" t="n">
-        <v>8.16</v>
+        <v>8.18</v>
       </c>
     </row>
     <row r="341">
@@ -11862,7 +11862,7 @@
         </is>
       </c>
       <c r="H341" s="1" t="n">
-        <v>40</v>
+        <v>39.92</v>
       </c>
     </row>
     <row r="342">
@@ -11895,7 +11895,7 @@
         </is>
       </c>
       <c r="H342" s="1" t="n">
-        <v>175.8</v>
+        <v>173.2</v>
       </c>
     </row>
     <row r="343">
@@ -11928,7 +11928,7 @@
         </is>
       </c>
       <c r="H343" s="1" t="n">
-        <v>16.19</v>
+        <v>16.01</v>
       </c>
     </row>
     <row r="344">
@@ -11961,7 +11961,7 @@
         </is>
       </c>
       <c r="H344" s="1" t="n">
-        <v>31.4</v>
+        <v>31.44</v>
       </c>
     </row>
     <row r="345">
@@ -11994,7 +11994,7 @@
         </is>
       </c>
       <c r="H345" s="1" t="n">
-        <v>4.71</v>
+        <v>4.72</v>
       </c>
     </row>
     <row r="346">
@@ -12027,7 +12027,7 @@
         </is>
       </c>
       <c r="H346" s="1" t="n">
-        <v>295.5</v>
+        <v>294.5</v>
       </c>
     </row>
     <row r="347">
@@ -12060,7 +12060,7 @@
         </is>
       </c>
       <c r="H347" s="1" t="n">
-        <v>5.08</v>
+        <v>5.09</v>
       </c>
     </row>
     <row r="348">
@@ -12093,7 +12093,7 @@
         </is>
       </c>
       <c r="H348" s="1" t="n">
-        <v>12.36</v>
+        <v>12.43</v>
       </c>
     </row>
     <row r="349">
@@ -12126,7 +12126,7 @@
         </is>
       </c>
       <c r="H349" s="1" t="n">
-        <v>57</v>
+        <v>57.2</v>
       </c>
     </row>
     <row r="350">
@@ -12192,7 +12192,7 @@
         </is>
       </c>
       <c r="H351" s="1" t="n">
-        <v>12.91</v>
+        <v>12.92</v>
       </c>
     </row>
     <row r="352">
@@ -12225,7 +12225,7 @@
         </is>
       </c>
       <c r="H352" s="1" t="n">
-        <v>10.08</v>
+        <v>10.12</v>
       </c>
     </row>
     <row r="353">
@@ -12291,7 +12291,7 @@
         </is>
       </c>
       <c r="H354" s="1" t="n">
-        <v>30.1</v>
+        <v>30.08</v>
       </c>
     </row>
     <row r="355">
@@ -12324,7 +12324,7 @@
         </is>
       </c>
       <c r="H355" s="1" t="n">
-        <v>24.76</v>
+        <v>24.42</v>
       </c>
     </row>
     <row r="356">
@@ -12357,7 +12357,7 @@
         </is>
       </c>
       <c r="H356" s="1" t="n">
-        <v>31.08</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="357">
@@ -12489,7 +12489,7 @@
         </is>
       </c>
       <c r="H360" s="1" t="n">
-        <v>40.96</v>
+        <v>40.66</v>
       </c>
     </row>
     <row r="361">
@@ -12555,7 +12555,7 @@
         </is>
       </c>
       <c r="H362" s="1" t="n">
-        <v>8.619999999999999</v>
+        <v>8.67</v>
       </c>
     </row>
     <row r="363">
@@ -12588,7 +12588,7 @@
         </is>
       </c>
       <c r="H363" s="1" t="n">
-        <v>123.2</v>
+        <v>123</v>
       </c>
     </row>
     <row r="364">
@@ -12621,7 +12621,7 @@
         </is>
       </c>
       <c r="H364" s="1" t="n">
-        <v>7.06</v>
+        <v>7.08</v>
       </c>
     </row>
     <row r="365">
@@ -12720,7 +12720,7 @@
         </is>
       </c>
       <c r="H367" s="1" t="n">
-        <v>21.98</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="368">
@@ -12753,7 +12753,7 @@
         </is>
       </c>
       <c r="H368" s="1" t="n">
-        <v>5.2</v>
+        <v>5.18</v>
       </c>
     </row>
     <row r="369">
@@ -12786,7 +12786,7 @@
         </is>
       </c>
       <c r="H369" s="1" t="n">
-        <v>242.8</v>
+        <v>242.3</v>
       </c>
     </row>
     <row r="370">
@@ -12819,7 +12819,7 @@
         </is>
       </c>
       <c r="H370" s="1" t="n">
-        <v>4.6</v>
+        <v>4.67</v>
       </c>
     </row>
     <row r="371">
@@ -12885,7 +12885,7 @@
         </is>
       </c>
       <c r="H372" s="1" t="n">
-        <v>8.619999999999999</v>
+        <v>8.609999999999999</v>
       </c>
     </row>
     <row r="373">
@@ -12905,7 +12905,7 @@
         </is>
       </c>
       <c r="D373" s="1" t="n">
-        <v>7.7754</v>
+        <v>7.836549</v>
       </c>
       <c r="F373" t="inlineStr">
         <is>
@@ -12938,7 +12938,7 @@
         </is>
       </c>
       <c r="D374" s="1" t="n">
-        <v>11.02387</v>
+        <v>10.977818</v>
       </c>
       <c r="F374" t="inlineStr">
         <is>
@@ -12984,7 +12984,7 @@
         </is>
       </c>
       <c r="H375" s="1" t="n">
-        <v>31.16</v>
+        <v>31.14</v>
       </c>
     </row>
     <row r="376">
@@ -13004,7 +13004,7 @@
         </is>
       </c>
       <c r="D376" s="1" t="n">
-        <v>17.723678</v>
+        <v>17.628156</v>
       </c>
       <c r="F376" t="inlineStr">
         <is>
@@ -13017,7 +13017,7 @@
         </is>
       </c>
       <c r="H376" s="1" t="n">
-        <v>8.91</v>
+        <v>8.880000000000001</v>
       </c>
     </row>
     <row r="377">
@@ -13050,7 +13050,7 @@
         </is>
       </c>
       <c r="H377" s="1" t="n">
-        <v>604</v>
+        <v>590</v>
       </c>
     </row>
     <row r="378">
@@ -13083,7 +13083,7 @@
         </is>
       </c>
       <c r="H378" s="1" t="n">
-        <v>5.4</v>
+        <v>5.43</v>
       </c>
     </row>
     <row r="379">
@@ -13116,7 +13116,7 @@
         </is>
       </c>
       <c r="H379" s="1" t="n">
-        <v>4.61</v>
+        <v>4.62</v>
       </c>
     </row>
     <row r="380">
@@ -13149,7 +13149,7 @@
         </is>
       </c>
       <c r="H380" s="1" t="n">
-        <v>8.83</v>
+        <v>8.779999999999999</v>
       </c>
     </row>
     <row r="381">
@@ -13182,7 +13182,7 @@
         </is>
       </c>
       <c r="H381" s="1" t="n">
-        <v>17.73</v>
+        <v>17.78</v>
       </c>
     </row>
     <row r="382">
@@ -13215,7 +13215,7 @@
         </is>
       </c>
       <c r="H382" s="1" t="n">
-        <v>111.5</v>
+        <v>111.4</v>
       </c>
     </row>
     <row r="383">
@@ -13248,7 +13248,7 @@
         </is>
       </c>
       <c r="H383" s="1" t="n">
-        <v>11.03</v>
+        <v>11.02</v>
       </c>
     </row>
     <row r="384">
@@ -13314,7 +13314,7 @@
         </is>
       </c>
       <c r="H385" s="1" t="n">
-        <v>4.5</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="386">
@@ -13334,7 +13334,7 @@
         </is>
       </c>
       <c r="D386" s="1" t="n">
-        <v>2.8489</v>
+        <v>2.860757</v>
       </c>
       <c r="F386" t="inlineStr">
         <is>
@@ -13347,7 +13347,7 @@
         </is>
       </c>
       <c r="H386" s="1" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="387">
@@ -13380,7 +13380,7 @@
         </is>
       </c>
       <c r="H387" s="1" t="n">
-        <v>300.25</v>
+        <v>302</v>
       </c>
     </row>
     <row r="388">
@@ -13446,7 +13446,7 @@
         </is>
       </c>
       <c r="H389" s="1" t="n">
-        <v>35.52</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="390">
@@ -13512,7 +13512,7 @@
         </is>
       </c>
       <c r="H391" s="1" t="n">
-        <v>52</v>
+        <v>52.1</v>
       </c>
     </row>
     <row r="392">
@@ -13578,7 +13578,7 @@
         </is>
       </c>
       <c r="H393" s="1" t="n">
-        <v>2.75</v>
+        <v>2.71</v>
       </c>
     </row>
     <row r="394">
@@ -13611,7 +13611,7 @@
         </is>
       </c>
       <c r="H394" s="1" t="n">
-        <v>108.6</v>
+        <v>108.2</v>
       </c>
     </row>
     <row r="395">
@@ -13677,7 +13677,7 @@
         </is>
       </c>
       <c r="H396" s="1" t="n">
-        <v>1.85</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="397">
@@ -13710,7 +13710,7 @@
         </is>
       </c>
       <c r="H397" s="1" t="n">
-        <v>170.1</v>
+        <v>169.6</v>
       </c>
     </row>
     <row r="398">
@@ -13743,7 +13743,7 @@
         </is>
       </c>
       <c r="H398" s="1" t="n">
-        <v>30.62</v>
+        <v>30.58</v>
       </c>
     </row>
     <row r="399">
@@ -13776,7 +13776,7 @@
         </is>
       </c>
       <c r="H399" s="1" t="n">
-        <v>13.16</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="400">
@@ -13809,7 +13809,7 @@
         </is>
       </c>
       <c r="H400" s="1" t="n">
-        <v>3.96</v>
+        <v>3.98</v>
       </c>
     </row>
     <row r="401">
@@ -13842,7 +13842,7 @@
         </is>
       </c>
       <c r="H401" s="1" t="n">
-        <v>17.22</v>
+        <v>17.19</v>
       </c>
     </row>
     <row r="402">
@@ -13875,7 +13875,7 @@
         </is>
       </c>
       <c r="H402" s="1" t="n">
-        <v>6.77</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="403">
@@ -13908,7 +13908,7 @@
         </is>
       </c>
       <c r="H403" s="1" t="n">
-        <v>14.96</v>
+        <v>14.87</v>
       </c>
     </row>
     <row r="404">
@@ -13941,7 +13941,7 @@
         </is>
       </c>
       <c r="H404" s="1" t="n">
-        <v>5.12</v>
+        <v>5.14</v>
       </c>
     </row>
     <row r="405">
@@ -14007,7 +14007,7 @@
         </is>
       </c>
       <c r="H406" s="1" t="n">
-        <v>5.77</v>
+        <v>5.76</v>
       </c>
     </row>
     <row r="407">
@@ -14040,7 +14040,7 @@
         </is>
       </c>
       <c r="H407" s="1" t="n">
-        <v>11.84</v>
+        <v>11.83</v>
       </c>
     </row>
     <row r="408">
@@ -14073,7 +14073,7 @@
         </is>
       </c>
       <c r="H408" s="1" t="n">
-        <v>28.58</v>
+        <v>28.62</v>
       </c>
     </row>
     <row r="409">
@@ -14139,7 +14139,7 @@
         </is>
       </c>
       <c r="H410" s="1" t="n">
-        <v>5.19</v>
+        <v>5.18</v>
       </c>
     </row>
     <row r="411">
@@ -14172,7 +14172,7 @@
         </is>
       </c>
       <c r="H411" s="1" t="n">
-        <v>1.56</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="412">
@@ -14205,7 +14205,7 @@
         </is>
       </c>
       <c r="H412" s="1" t="n">
-        <v>20.14</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="413">
@@ -14238,7 +14238,7 @@
         </is>
       </c>
       <c r="H413" s="1" t="n">
-        <v>3.73</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="414">
@@ -14291,7 +14291,7 @@
         </is>
       </c>
       <c r="D415" s="1" t="n">
-        <v>0</v>
+        <v>19.684179</v>
       </c>
       <c r="F415" t="inlineStr">
         <is>
@@ -14304,7 +14304,7 @@
         </is>
       </c>
       <c r="H415" s="1" t="n">
-        <v>3.66</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="416">
@@ -14337,7 +14337,7 @@
         </is>
       </c>
       <c r="H416" s="1" t="n">
-        <v>7.56</v>
+        <v>7.55</v>
       </c>
     </row>
     <row r="417">
@@ -14370,7 +14370,7 @@
         </is>
       </c>
       <c r="H417" s="1" t="n">
-        <v>9.220000000000001</v>
+        <v>9.210000000000001</v>
       </c>
     </row>
     <row r="418">
@@ -14403,7 +14403,7 @@
         </is>
       </c>
       <c r="H418" s="1" t="n">
-        <v>11.76</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="419">
@@ -14436,7 +14436,7 @@
         </is>
       </c>
       <c r="H419" s="1" t="n">
-        <v>18.76</v>
+        <v>18.73</v>
       </c>
     </row>
     <row r="420">
@@ -14469,7 +14469,7 @@
         </is>
       </c>
       <c r="H420" s="1" t="n">
-        <v>30.8</v>
+        <v>30.68</v>
       </c>
     </row>
     <row r="421">
@@ -14489,7 +14489,7 @@
         </is>
       </c>
       <c r="D421" s="1" t="n">
-        <v>3.919713</v>
+        <v>3.91902</v>
       </c>
       <c r="F421" t="inlineStr">
         <is>
@@ -14502,7 +14502,7 @@
         </is>
       </c>
       <c r="H421" s="1" t="n">
-        <v>75.90000000000001</v>
+        <v>76.09999999999999</v>
       </c>
     </row>
     <row r="422">
@@ -14535,7 +14535,7 @@
         </is>
       </c>
       <c r="H422" s="1" t="n">
-        <v>44.02</v>
+        <v>43.78</v>
       </c>
     </row>
     <row r="423">
@@ -14601,7 +14601,7 @@
         </is>
       </c>
       <c r="H424" s="1" t="n">
-        <v>34.66</v>
+        <v>34.52</v>
       </c>
     </row>
     <row r="425">
@@ -14667,7 +14667,7 @@
         </is>
       </c>
       <c r="H426" s="1" t="n">
-        <v>10.7</v>
+        <v>10.85</v>
       </c>
     </row>
     <row r="427">
@@ -14700,7 +14700,7 @@
         </is>
       </c>
       <c r="H427" s="1" t="n">
-        <v>8.92</v>
+        <v>9.02</v>
       </c>
     </row>
     <row r="428">
@@ -14733,7 +14733,7 @@
         </is>
       </c>
       <c r="H428" s="1" t="n">
-        <v>25.38</v>
+        <v>25.42</v>
       </c>
     </row>
     <row r="429">
@@ -14799,7 +14799,7 @@
         </is>
       </c>
       <c r="H430" s="1" t="n">
-        <v>5.5</v>
+        <v>5.51</v>
       </c>
     </row>
     <row r="431">
@@ -14832,7 +14832,7 @@
         </is>
       </c>
       <c r="H431" s="1" t="n">
-        <v>4.14</v>
+        <v>4.16</v>
       </c>
     </row>
     <row r="432">
@@ -14865,7 +14865,7 @@
         </is>
       </c>
       <c r="H432" s="1" t="n">
-        <v>19.08</v>
+        <v>19.27</v>
       </c>
     </row>
     <row r="433">
@@ -14898,7 +14898,7 @@
         </is>
       </c>
       <c r="H433" s="1" t="n">
-        <v>49.04</v>
+        <v>49.08</v>
       </c>
     </row>
     <row r="434">
@@ -14964,7 +14964,7 @@
         </is>
       </c>
       <c r="H435" s="1" t="n">
-        <v>31.08</v>
+        <v>30.86</v>
       </c>
     </row>
     <row r="436">
@@ -14997,7 +14997,7 @@
         </is>
       </c>
       <c r="H436" s="1" t="n">
-        <v>10.59</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="437">
@@ -15030,7 +15030,7 @@
         </is>
       </c>
       <c r="H437" s="1" t="n">
-        <v>78.34999999999999</v>
+        <v>78.09999999999999</v>
       </c>
     </row>
     <row r="438">
@@ -15063,7 +15063,7 @@
         </is>
       </c>
       <c r="H438" s="1" t="n">
-        <v>11.1</v>
+        <v>11.15</v>
       </c>
     </row>
     <row r="439">
@@ -15129,7 +15129,7 @@
         </is>
       </c>
       <c r="H440" s="1" t="n">
-        <v>211</v>
+        <v>209.5</v>
       </c>
     </row>
     <row r="441">
@@ -15162,7 +15162,7 @@
         </is>
       </c>
       <c r="H441" s="1" t="n">
-        <v>13.01</v>
+        <v>13.07</v>
       </c>
     </row>
     <row r="442">
@@ -15195,7 +15195,7 @@
         </is>
       </c>
       <c r="H442" s="1" t="n">
-        <v>12.36</v>
+        <v>12.41</v>
       </c>
     </row>
     <row r="443">
@@ -15215,7 +15215,7 @@
         </is>
       </c>
       <c r="D443" s="1" t="n">
-        <v>2.377489</v>
+        <v>2.37701</v>
       </c>
       <c r="F443" t="inlineStr">
         <is>
@@ -15228,7 +15228,7 @@
         </is>
       </c>
       <c r="H443" s="1" t="n">
-        <v>40.7</v>
+        <v>40.6</v>
       </c>
     </row>
     <row r="444">
@@ -15261,7 +15261,7 @@
         </is>
       </c>
       <c r="H444" s="1" t="n">
-        <v>20.08</v>
+        <v>20.1</v>
       </c>
     </row>
     <row r="445">
@@ -15327,7 +15327,7 @@
         </is>
       </c>
       <c r="H446" s="1" t="n">
-        <v>9.01</v>
+        <v>9.06</v>
       </c>
     </row>
     <row r="447">
@@ -15360,7 +15360,7 @@
         </is>
       </c>
       <c r="H447" s="1" t="n">
-        <v>7.67</v>
+        <v>7.66</v>
       </c>
     </row>
     <row r="448">
@@ -15393,7 +15393,7 @@
         </is>
       </c>
       <c r="H448" s="1" t="n">
-        <v>5.59</v>
+        <v>5.58</v>
       </c>
     </row>
     <row r="449">
@@ -15426,7 +15426,7 @@
         </is>
       </c>
       <c r="H449" s="1" t="n">
-        <v>9.029999999999999</v>
+        <v>9.01</v>
       </c>
     </row>
     <row r="450">
@@ -15459,7 +15459,7 @@
         </is>
       </c>
       <c r="H450" s="1" t="n">
-        <v>145.5</v>
+        <v>145.6</v>
       </c>
     </row>
     <row r="451">
@@ -15492,7 +15492,7 @@
         </is>
       </c>
       <c r="H451" s="1" t="n">
-        <v>1.19</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="452">
@@ -15525,7 +15525,7 @@
         </is>
       </c>
       <c r="H452" s="1" t="n">
-        <v>6.86</v>
+        <v>6.89</v>
       </c>
     </row>
     <row r="453">
@@ -15558,7 +15558,7 @@
         </is>
       </c>
       <c r="H453" s="1" t="n">
-        <v>35</v>
+        <v>34.98</v>
       </c>
     </row>
     <row r="454">
@@ -15591,7 +15591,7 @@
         </is>
       </c>
       <c r="H454" s="1" t="n">
-        <v>13.86</v>
+        <v>13.79</v>
       </c>
     </row>
     <row r="455">
@@ -15624,7 +15624,7 @@
         </is>
       </c>
       <c r="H455" s="1" t="n">
-        <v>10.15</v>
+        <v>10.13</v>
       </c>
     </row>
     <row r="456">
@@ -15657,7 +15657,7 @@
         </is>
       </c>
       <c r="H456" s="1" t="n">
-        <v>41.1</v>
+        <v>41</v>
       </c>
     </row>
     <row r="457">
@@ -15690,7 +15690,7 @@
         </is>
       </c>
       <c r="H457" s="1" t="n">
-        <v>1617</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="458">
@@ -15723,7 +15723,7 @@
         </is>
       </c>
       <c r="H458" s="1" t="n">
-        <v>3.47</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="459">
@@ -15822,7 +15822,7 @@
         </is>
       </c>
       <c r="H461" s="1" t="n">
-        <v>12.11</v>
+        <v>12.06</v>
       </c>
     </row>
     <row r="462">
@@ -15921,7 +15921,7 @@
         </is>
       </c>
       <c r="H464" s="1" t="n">
-        <v>31.78</v>
+        <v>31.92</v>
       </c>
     </row>
     <row r="465">
@@ -15954,7 +15954,7 @@
         </is>
       </c>
       <c r="H465" s="1" t="n">
-        <v>18.04</v>
+        <v>18.07</v>
       </c>
     </row>
     <row r="466">
@@ -15987,7 +15987,7 @@
         </is>
       </c>
       <c r="H466" s="1" t="n">
-        <v>3.31</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="467">
@@ -16020,7 +16020,7 @@
         </is>
       </c>
       <c r="H467" s="1" t="n">
-        <v>37.78</v>
+        <v>37.82</v>
       </c>
     </row>
     <row r="468">
@@ -16086,7 +16086,7 @@
         </is>
       </c>
       <c r="H469" s="1" t="n">
-        <v>5.62</v>
+        <v>5.68</v>
       </c>
     </row>
     <row r="470">
@@ -16119,7 +16119,7 @@
         </is>
       </c>
       <c r="H470" s="1" t="n">
-        <v>12.48</v>
+        <v>12.47</v>
       </c>
     </row>
     <row r="471">
@@ -16152,7 +16152,7 @@
         </is>
       </c>
       <c r="H471" s="1" t="n">
-        <v>87.55</v>
+        <v>87.09999999999999</v>
       </c>
     </row>
     <row r="472">
@@ -16185,7 +16185,7 @@
         </is>
       </c>
       <c r="H472" s="1" t="n">
-        <v>109.8</v>
+        <v>110.8</v>
       </c>
     </row>
     <row r="473">
@@ -16251,7 +16251,7 @@
         </is>
       </c>
       <c r="H474" s="1" t="n">
-        <v>16.84</v>
+        <v>17.04</v>
       </c>
     </row>
     <row r="475">
@@ -16284,7 +16284,7 @@
         </is>
       </c>
       <c r="H475" s="1" t="n">
-        <v>9.210000000000001</v>
+        <v>9.24</v>
       </c>
     </row>
     <row r="476">
@@ -16317,7 +16317,7 @@
         </is>
       </c>
       <c r="H476" s="1" t="n">
-        <v>5.29</v>
+        <v>5.24</v>
       </c>
     </row>
     <row r="477">
@@ -16383,7 +16383,7 @@
         </is>
       </c>
       <c r="H478" s="1" t="n">
-        <v>4.91</v>
+        <v>4.95</v>
       </c>
     </row>
     <row r="479">
@@ -16416,7 +16416,7 @@
         </is>
       </c>
       <c r="H479" s="1" t="n">
-        <v>64.25</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="480">
@@ -16449,7 +16449,7 @@
         </is>
       </c>
       <c r="H480" s="1" t="n">
-        <v>6.84</v>
+        <v>6.82</v>
       </c>
     </row>
     <row r="481">
@@ -16515,7 +16515,7 @@
         </is>
       </c>
       <c r="H482" s="1" t="n">
-        <v>4.37</v>
+        <v>4.32</v>
       </c>
     </row>
     <row r="483">
@@ -16548,7 +16548,7 @@
         </is>
       </c>
       <c r="H483" s="1" t="n">
-        <v>28.32</v>
+        <v>28.04</v>
       </c>
     </row>
     <row r="484">
@@ -16581,7 +16581,7 @@
         </is>
       </c>
       <c r="H484" s="1" t="n">
-        <v>2.9</v>
+        <v>2.89</v>
       </c>
     </row>
     <row r="485">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="H485" s="1" t="n">
-        <v>13.64</v>
+        <v>13.55</v>
       </c>
     </row>
     <row r="486">
@@ -16647,7 +16647,7 @@
         </is>
       </c>
       <c r="H486" s="1" t="n">
-        <v>81.90000000000001</v>
+        <v>81.65000000000001</v>
       </c>
     </row>
     <row r="487">
@@ -16680,7 +16680,7 @@
         </is>
       </c>
       <c r="H487" s="1" t="n">
-        <v>35.12</v>
+        <v>34.86</v>
       </c>
     </row>
     <row r="488">
@@ -16713,7 +16713,7 @@
         </is>
       </c>
       <c r="H488" s="1" t="n">
-        <v>22.8</v>
+        <v>22.82</v>
       </c>
     </row>
     <row r="489">
@@ -16779,7 +16779,7 @@
         </is>
       </c>
       <c r="H490" s="1" t="n">
-        <v>27.6</v>
+        <v>27.64</v>
       </c>
     </row>
     <row r="491">
@@ -16812,7 +16812,7 @@
         </is>
       </c>
       <c r="H491" s="1" t="n">
-        <v>87.2</v>
+        <v>87</v>
       </c>
     </row>
     <row r="492">
@@ -16845,7 +16845,7 @@
         </is>
       </c>
       <c r="H492" s="1" t="n">
-        <v>7.25</v>
+        <v>7.28</v>
       </c>
     </row>
     <row r="493">
@@ -16878,7 +16878,7 @@
         </is>
       </c>
       <c r="H493" s="1" t="n">
-        <v>29.74</v>
+        <v>29.7</v>
       </c>
     </row>
     <row r="494">
@@ -16977,7 +16977,7 @@
         </is>
       </c>
       <c r="H496" s="1" t="n">
-        <v>2.92</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="497">
@@ -17043,7 +17043,7 @@
         </is>
       </c>
       <c r="H498" s="1" t="n">
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
     </row>
     <row r="499">
@@ -17109,7 +17109,7 @@
         </is>
       </c>
       <c r="H500" s="1" t="n">
-        <v>2.08</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="501">
@@ -17142,7 +17142,7 @@
         </is>
       </c>
       <c r="H501" s="1" t="n">
-        <v>13.82</v>
+        <v>13.72</v>
       </c>
     </row>
     <row r="502">
@@ -17175,7 +17175,7 @@
         </is>
       </c>
       <c r="H502" s="1" t="n">
-        <v>7.77</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="503">
@@ -17208,7 +17208,7 @@
         </is>
       </c>
       <c r="H503" s="1" t="n">
-        <v>24.58</v>
+        <v>24.56</v>
       </c>
     </row>
     <row r="504">
@@ -17340,7 +17340,7 @@
         </is>
       </c>
       <c r="H507" s="1" t="n">
-        <v>2.22</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="508">
@@ -17373,7 +17373,7 @@
         </is>
       </c>
       <c r="H508" s="1" t="n">
-        <v>12.71</v>
+        <v>12.72</v>
       </c>
     </row>
     <row r="509">
@@ -17406,7 +17406,7 @@
         </is>
       </c>
       <c r="H509" s="1" t="n">
-        <v>9.52</v>
+        <v>9.460000000000001</v>
       </c>
     </row>
     <row r="510">
@@ -17472,7 +17472,7 @@
         </is>
       </c>
       <c r="H511" s="1" t="n">
-        <v>17.36</v>
+        <v>17.55</v>
       </c>
     </row>
     <row r="512">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="H515" s="1" t="n">
-        <v>2.46</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="516">
@@ -17657,7 +17657,7 @@
         </is>
       </c>
       <c r="D517" s="1" t="n">
-        <v>2.219586</v>
+        <v>2.226768</v>
       </c>
       <c r="F517" t="inlineStr">
         <is>
@@ -17670,7 +17670,7 @@
         </is>
       </c>
       <c r="H517" s="1" t="n">
-        <v>9.43</v>
+        <v>9.390000000000001</v>
       </c>
     </row>
     <row r="518">
@@ -17703,7 +17703,7 @@
         </is>
       </c>
       <c r="H518" s="1" t="n">
-        <v>26.24</v>
+        <v>25.98</v>
       </c>
     </row>
     <row r="519">
@@ -17835,7 +17835,7 @@
         </is>
       </c>
       <c r="H522" s="1" t="n">
-        <v>24.74</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="523">
@@ -17868,7 +17868,7 @@
         </is>
       </c>
       <c r="H523" s="1" t="n">
-        <v>2.27</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="524">
@@ -17967,7 +17967,7 @@
         </is>
       </c>
       <c r="H526" s="1" t="n">
-        <v>8.710000000000001</v>
+        <v>8.73</v>
       </c>
     </row>
     <row r="527">
@@ -18000,7 +18000,7 @@
         </is>
       </c>
       <c r="H527" s="1" t="n">
-        <v>1.45</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="528">
@@ -18033,7 +18033,7 @@
         </is>
       </c>
       <c r="H528" s="1" t="n">
-        <v>78.8</v>
+        <v>78.40000000000001</v>
       </c>
     </row>
     <row r="529">
@@ -18066,7 +18066,7 @@
         </is>
       </c>
       <c r="H529" s="1" t="n">
-        <v>1.76</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="530">
@@ -18099,7 +18099,7 @@
         </is>
       </c>
       <c r="H530" s="1" t="n">
-        <v>9.220000000000001</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="531">
@@ -18132,7 +18132,7 @@
         </is>
       </c>
       <c r="H531" s="1" t="n">
-        <v>14.52</v>
+        <v>14.53</v>
       </c>
     </row>
     <row r="532">
@@ -18165,7 +18165,7 @@
         </is>
       </c>
       <c r="H532" s="1" t="n">
-        <v>35.36</v>
+        <v>35.24</v>
       </c>
     </row>
     <row r="533">
@@ -18198,7 +18198,7 @@
         </is>
       </c>
       <c r="H533" s="1" t="n">
-        <v>1.52</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="534">
@@ -18231,7 +18231,7 @@
         </is>
       </c>
       <c r="H534" s="1" t="n">
-        <v>8.140000000000001</v>
+        <v>8.08</v>
       </c>
     </row>
     <row r="535">
@@ -18264,7 +18264,7 @@
         </is>
       </c>
       <c r="H535" s="1" t="n">
-        <v>3.25</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="536">
@@ -18297,7 +18297,7 @@
         </is>
       </c>
       <c r="H536" s="1" t="n">
-        <v>158.8</v>
+        <v>159</v>
       </c>
     </row>
     <row r="537">
@@ -18330,7 +18330,7 @@
         </is>
       </c>
       <c r="H537" s="1" t="n">
-        <v>2.61</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="538">
@@ -18363,7 +18363,7 @@
         </is>
       </c>
       <c r="H538" s="1" t="n">
-        <v>6.41</v>
+        <v>6.42</v>
       </c>
     </row>
     <row r="539">
@@ -18396,7 +18396,7 @@
         </is>
       </c>
       <c r="H539" s="1" t="n">
-        <v>7.99</v>
+        <v>8.01</v>
       </c>
     </row>
     <row r="540">
@@ -18429,7 +18429,7 @@
         </is>
       </c>
       <c r="H540" s="1" t="n">
-        <v>72.40000000000001</v>
+        <v>71.75</v>
       </c>
     </row>
     <row r="541">
@@ -18462,7 +18462,7 @@
         </is>
       </c>
       <c r="H541" s="1" t="n">
-        <v>27.5</v>
+        <v>27.56</v>
       </c>
     </row>
     <row r="542">
@@ -18528,7 +18528,7 @@
         </is>
       </c>
       <c r="H543" s="1" t="n">
-        <v>6.24</v>
+        <v>6.23</v>
       </c>
     </row>
     <row r="544">
@@ -18561,7 +18561,7 @@
         </is>
       </c>
       <c r="H544" s="1" t="n">
-        <v>21.46</v>
+        <v>21.68</v>
       </c>
     </row>
     <row r="545">
@@ -18627,7 +18627,7 @@
         </is>
       </c>
       <c r="H546" s="1" t="n">
-        <v>1.78</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="547">
@@ -18759,7 +18759,7 @@
         </is>
       </c>
       <c r="H550" s="1" t="n">
-        <v>3.85</v>
+        <v>3.88</v>
       </c>
     </row>
     <row r="551">
@@ -18858,7 +18858,7 @@
         </is>
       </c>
       <c r="H553" s="1" t="n">
-        <v>6.91</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="554">
@@ -18891,7 +18891,7 @@
         </is>
       </c>
       <c r="H554" s="1" t="n">
-        <v>3.88</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="555">
@@ -18924,7 +18924,7 @@
         </is>
       </c>
       <c r="H555" s="1" t="n">
-        <v>11.44</v>
+        <v>11.43</v>
       </c>
     </row>
     <row r="556">
@@ -18957,7 +18957,7 @@
         </is>
       </c>
       <c r="H556" s="1" t="n">
-        <v>12.56</v>
+        <v>12.38</v>
       </c>
     </row>
     <row r="557">
@@ -19023,7 +19023,7 @@
         </is>
       </c>
       <c r="H558" s="1" t="n">
-        <v>1.64</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="559">
@@ -19056,7 +19056,7 @@
         </is>
       </c>
       <c r="H559" s="1" t="n">
-        <v>7.41</v>
+        <v>7.45</v>
       </c>
     </row>
     <row r="560">
@@ -19089,7 +19089,7 @@
         </is>
       </c>
       <c r="H560" s="1" t="n">
-        <v>34.8</v>
+        <v>34.62</v>
       </c>
     </row>
     <row r="561">
@@ -19122,7 +19122,7 @@
         </is>
       </c>
       <c r="H561" s="1" t="n">
-        <v>27.08</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="562">
@@ -19155,7 +19155,7 @@
         </is>
       </c>
       <c r="H562" s="1" t="n">
-        <v>15.18</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="563">
@@ -19188,7 +19188,7 @@
         </is>
       </c>
       <c r="H563" s="1" t="n">
-        <v>29.3</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="564">
@@ -19221,7 +19221,7 @@
         </is>
       </c>
       <c r="H564" s="1" t="n">
-        <v>13.67</v>
+        <v>13.58</v>
       </c>
     </row>
     <row r="565">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="H565" s="1" t="n">
-        <v>19.2</v>
+        <v>19.24</v>
       </c>
     </row>
     <row r="566">
@@ -19287,7 +19287,7 @@
         </is>
       </c>
       <c r="H566" s="1" t="n">
-        <v>7.36</v>
+        <v>7.38</v>
       </c>
     </row>
     <row r="567">
@@ -19320,7 +19320,7 @@
         </is>
       </c>
       <c r="H567" s="1" t="n">
-        <v>111.2</v>
+        <v>111.3</v>
       </c>
     </row>
     <row r="568">
@@ -19386,7 +19386,7 @@
         </is>
       </c>
       <c r="H569" s="1" t="n">
-        <v>4.23</v>
+        <v>4.25</v>
       </c>
     </row>
     <row r="570">
@@ -19419,7 +19419,7 @@
         </is>
       </c>
       <c r="H570" s="1" t="n">
-        <v>11.73</v>
+        <v>12.11</v>
       </c>
     </row>
     <row r="571">
@@ -19485,7 +19485,7 @@
         </is>
       </c>
       <c r="H572" s="1" t="n">
-        <v>21.8</v>
+        <v>21.76</v>
       </c>
     </row>
     <row r="573">
@@ -19551,7 +19551,7 @@
         </is>
       </c>
       <c r="H574" s="1" t="n">
-        <v>143.8</v>
+        <v>143.9</v>
       </c>
     </row>
     <row r="575">
@@ -19584,7 +19584,7 @@
         </is>
       </c>
       <c r="H575" s="1" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="576">
@@ -19617,7 +19617,7 @@
         </is>
       </c>
       <c r="H576" s="1" t="n">
-        <v>4.1</v>
+        <v>4.11</v>
       </c>
     </row>
     <row r="577">
@@ -19650,7 +19650,7 @@
         </is>
       </c>
       <c r="H577" s="1" t="n">
-        <v>1.3</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="578">
@@ -19683,7 +19683,7 @@
         </is>
       </c>
       <c r="H578" s="1" t="n">
-        <v>127</v>
+        <v>127.5</v>
       </c>
     </row>
     <row r="579">
@@ -19815,7 +19815,7 @@
         </is>
       </c>
       <c r="H582" s="1" t="n">
-        <v>39.72</v>
+        <v>39.68</v>
       </c>
     </row>
     <row r="583">
@@ -19848,7 +19848,7 @@
         </is>
       </c>
       <c r="H583" s="1" t="n">
-        <v>1.53</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="584">
@@ -19881,7 +19881,7 @@
         </is>
       </c>
       <c r="H584" s="1" t="n">
-        <v>4.37</v>
+        <v>4.44</v>
       </c>
     </row>
     <row r="585">
@@ -19947,7 +19947,7 @@
         </is>
       </c>
       <c r="H586" s="1" t="n">
-        <v>14.36</v>
+        <v>14.1</v>
       </c>
     </row>
     <row r="587">
@@ -19980,7 +19980,7 @@
         </is>
       </c>
       <c r="H587" s="1" t="n">
-        <v>20.38</v>
+        <v>20.46</v>
       </c>
     </row>
     <row r="588">
@@ -20013,7 +20013,7 @@
         </is>
       </c>
       <c r="H588" s="1" t="n">
-        <v>48.62</v>
+        <v>48.6</v>
       </c>
     </row>
     <row r="589">
@@ -20046,7 +20046,7 @@
         </is>
       </c>
       <c r="H589" s="1" t="n">
-        <v>14.12</v>
+        <v>14.04</v>
       </c>
     </row>
     <row r="590">
@@ -20079,7 +20079,7 @@
         </is>
       </c>
       <c r="H590" s="1" t="n">
-        <v>47.58</v>
+        <v>49</v>
       </c>
     </row>
     <row r="591">
@@ -20145,7 +20145,7 @@
         </is>
       </c>
       <c r="H592" s="1" t="n">
-        <v>40.46</v>
+        <v>40.86</v>
       </c>
     </row>
     <row r="593">
@@ -20178,7 +20178,7 @@
         </is>
       </c>
       <c r="H593" s="1" t="n">
-        <v>5.72</v>
+        <v>5.78</v>
       </c>
     </row>
     <row r="594">
@@ -20211,7 +20211,7 @@
         </is>
       </c>
       <c r="H594" s="1" t="n">
-        <v>22.18</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="595">
@@ -20244,7 +20244,7 @@
         </is>
       </c>
       <c r="H595" s="1" t="n">
-        <v>3.34</v>
+        <v>3.36</v>
       </c>
     </row>
     <row r="596">
@@ -20277,7 +20277,7 @@
         </is>
       </c>
       <c r="H596" s="1" t="n">
-        <v>12.87</v>
+        <v>12.84</v>
       </c>
     </row>
     <row r="597">
@@ -20310,7 +20310,7 @@
         </is>
       </c>
       <c r="H597" s="1" t="n">
-        <v>112.6</v>
+        <v>114.4</v>
       </c>
     </row>
     <row r="598">
@@ -20442,7 +20442,7 @@
         </is>
       </c>
       <c r="H601" s="1" t="n">
-        <v>7.8</v>
+        <v>7.78</v>
       </c>
     </row>
     <row r="602">
@@ -20475,7 +20475,7 @@
         </is>
       </c>
       <c r="H602" s="1" t="n">
-        <v>21.98</v>
+        <v>22</v>
       </c>
     </row>
     <row r="603">
@@ -20508,7 +20508,7 @@
         </is>
       </c>
       <c r="H603" s="1" t="n">
-        <v>2.08</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="604">
@@ -20541,7 +20541,7 @@
         </is>
       </c>
       <c r="H604" s="1" t="n">
-        <v>22.44</v>
+        <v>22.42</v>
       </c>
     </row>
     <row r="605">
@@ -20574,7 +20574,7 @@
         </is>
       </c>
       <c r="H605" s="1" t="n">
-        <v>2.3</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="606">
@@ -20607,7 +20607,7 @@
         </is>
       </c>
       <c r="H606" s="1" t="n">
-        <v>23.2</v>
+        <v>23</v>
       </c>
     </row>
     <row r="607">
@@ -20673,7 +20673,7 @@
         </is>
       </c>
       <c r="H608" s="1" t="n">
-        <v>6</v>
+        <v>5.89</v>
       </c>
     </row>
     <row r="609">
@@ -20706,7 +20706,7 @@
         </is>
       </c>
       <c r="H609" s="1" t="n">
-        <v>6.89</v>
+        <v>6.86</v>
       </c>
     </row>
     <row r="610">
@@ -20772,7 +20772,7 @@
         </is>
       </c>
       <c r="H611" s="1" t="n">
-        <v>12.68</v>
+        <v>12.69</v>
       </c>
     </row>
     <row r="612">
@@ -20805,7 +20805,7 @@
         </is>
       </c>
       <c r="H612" s="1" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="613">
@@ -20838,7 +20838,7 @@
         </is>
       </c>
       <c r="H613" s="1" t="n">
-        <v>2.1</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="614">
@@ -20871,7 +20871,7 @@
         </is>
       </c>
       <c r="H614" s="1" t="n">
-        <v>21.72</v>
+        <v>21.54</v>
       </c>
     </row>
     <row r="615">
@@ -20937,7 +20937,7 @@
         </is>
       </c>
       <c r="H616" s="1" t="n">
-        <v>13</v>
+        <v>13.17</v>
       </c>
     </row>
     <row r="617">
@@ -20970,7 +20970,7 @@
         </is>
       </c>
       <c r="H617" s="1" t="n">
-        <v>10.13</v>
+        <v>10.15</v>
       </c>
     </row>
     <row r="618">
@@ -21036,7 +21036,7 @@
         </is>
       </c>
       <c r="H619" s="1" t="n">
-        <v>2.87</v>
+        <v>2.89</v>
       </c>
     </row>
     <row r="620">
@@ -21069,7 +21069,7 @@
         </is>
       </c>
       <c r="H620" s="1" t="n">
-        <v>8.91</v>
+        <v>8.98</v>
       </c>
     </row>
     <row r="621">
@@ -21102,7 +21102,7 @@
         </is>
       </c>
       <c r="H621" s="1" t="n">
-        <v>6.4</v>
+        <v>6.59</v>
       </c>
     </row>
     <row r="622">
@@ -21168,7 +21168,7 @@
         </is>
       </c>
       <c r="H623" s="1" t="n">
-        <v>4.73</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="624">
@@ -21234,7 +21234,7 @@
         </is>
       </c>
       <c r="H625" s="1" t="n">
-        <v>17.73</v>
+        <v>17.71</v>
       </c>
     </row>
     <row r="626">
@@ -21258,16 +21258,16 @@
       </c>
       <c r="F626" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>BETAE</t>
         </is>
       </c>
       <c r="G626" t="inlineStr">
         <is>
-          <t>DARPHANE ALTIN SERTİFİKASI</t>
+          <t>Beta Enerji ve Teknoloji AS</t>
         </is>
       </c>
       <c r="H626" s="1" t="n">
-        <v>73.59999999999999</v>
+        <v>83.84999999999999</v>
       </c>
     </row>
     <row r="627">
@@ -21291,16 +21291,16 @@
       </c>
       <c r="F627" t="inlineStr">
         <is>
-          <t>ORZAX</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="G627" t="inlineStr">
         <is>
-          <t>Orzaks Ilac ve Kimya Sanayi Ticaret A.S.</t>
+          <t>Agaoglu Avrasya Gayrimenkul Yatirim Ortakligi AS</t>
         </is>
       </c>
       <c r="H627" s="1" t="n">
-        <v>87.05</v>
+        <v>11.91</v>
       </c>
     </row>
     <row r="628">
@@ -21324,16 +21324,16 @@
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>ORZAX</t>
         </is>
       </c>
       <c r="G628" t="inlineStr">
         <is>
-          <t>Enpara Bank A.S.</t>
+          <t>Orzaks Ilac ve Kimya Sanayi Ticaret A.S.</t>
         </is>
       </c>
       <c r="H628" s="1" t="n">
-        <v>53.7</v>
+        <v>86.59999999999999</v>
       </c>
     </row>
     <row r="629">
@@ -21357,16 +21357,16 @@
       </c>
       <c r="F629" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="G629" t="inlineStr">
         <is>
-          <t>Agaoglu Avrasya Gayrimenkul Yatirim Ortakligi AS</t>
+          <t>DARPHANE ALTIN SERTİFİKASI</t>
         </is>
       </c>
       <c r="H629" s="1" t="n">
-        <v>11.93</v>
+        <v>73.48</v>
       </c>
     </row>
     <row r="630">
@@ -21390,16 +21390,16 @@
       </c>
       <c r="F630" t="inlineStr">
         <is>
-          <t>BETAE</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="G630" t="inlineStr">
         <is>
-          <t>Beta Enerji ve Teknoloji AS</t>
+          <t>Enpara Bank A.S.</t>
         </is>
       </c>
       <c r="H630" s="1" t="n">
-        <v>83.95</v>
+        <v>53.7</v>
       </c>
     </row>
     <row r="631">

</xml_diff>